<commit_message>
Update NFL production artifacts
</commit_message>
<xml_diff>
--- a/nfl-backend/data_delivery/nfl_feature_workbook_2026-09-24.xlsx
+++ b/nfl-backend/data_delivery/nfl_feature_workbook_2026-09-24.xlsx
@@ -8,9 +8,17 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFE Run Detail" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per-Fold Detail" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Pool" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Features (Master)" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Production (23)" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Candidates" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RFE Run Detail" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Per-Fold Detail" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Redundancy" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Coverage Gaps" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Glossary" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature Pool" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -61,7 +69,7 @@
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="top" wrapText="1"/>
+      <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -433,106 +441,1921 @@
   </sheetPr>
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>NFL Feature Selection Decision Workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Trace</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>nfl_feature_selection_20260924.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Run mode</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>full_history</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Production width before run</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Pool size</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Trials scored</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Committed trials</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Selected columns (record-only)</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>elo_diff, win_pct_diff, rest_days_diff, is_dome_home, ewm_net_pts_diff, ewm_ypp_diff, pace_plays_min_diff, rest_short_diff, div_game, travel_miles_diff, altitude_home, prime_time, elo_home, elo_away, win_pct_home, win_pct_away, ewm_net_pts_home, ewm_net_pts_away, ewm_ypp_home, ewm_ypp_away, rest_days_home, rest_days_away, is_home</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Default governance: this workbook does not change production. Adoption is explicit.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C00000"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="48" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>NFL Feature Selection Decision Workbook</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="n"/>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Non-null games</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Coverage %</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Scored rows</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Trace</t>
+          <t>ewm_ypp_diff</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>nfl_feature_selection_20260924.json</t>
-        </is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="n">
+        <v>2111</v>
+      </c>
+      <c r="E2" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="F2" s="2" t="n">
+        <v>2159</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Run mode</t>
+          <t>pace_plays_min_diff</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>full_history</t>
-        </is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="n">
+        <v>2111</v>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>97.78</v>
+      </c>
+      <c r="F3" s="2" t="n">
+        <v>2159</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Production width before run</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="n">
-        <v>23</v>
+          <t>is_dome_home</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="n">
+        <v>2118</v>
+      </c>
+      <c r="E4" s="2" t="n">
+        <v>98.09999999999999</v>
+      </c>
+      <c r="F4" s="2" t="n">
+        <v>2159</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Pool size</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>23</v>
+          <t>ewm_ypp_away</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="n">
+        <v>2126</v>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>98.47</v>
+      </c>
+      <c r="F5" s="2" t="n">
+        <v>2159</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Trials scored</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>23</v>
+          <t>ewm_ypp_home</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n">
+        <v>2128</v>
+      </c>
+      <c r="E6" s="2" t="n">
+        <v>98.56</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>2159</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Committed trials</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>0</v>
+          <t>win_pct_diff</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>2142</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>2159</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Selected columns (record-only)</t>
+          <t>rest_days_diff</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>elo_diff, win_pct_diff, rest_days_diff, is_dome_home, ewm_net_pts_diff, ewm_ypp_diff, pace_plays_min_diff, rest_short_diff, div_game, travel_miles_diff, altitude_home, prime_time, elo_home, elo_away, win_pct_home, win_pct_away, ewm_net_pts_home, ewm_net_pts_away, ewm_ypp_home, ewm_ypp_away, rest_days_home, rest_days_away, is_home</t>
-        </is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>2142</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>2159</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_diff</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>2142</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>2159</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Default governance: this workbook does not change production. Adoption is explicit.</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="n"/>
+          <t>rest_short_diff</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>2142</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_away</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="n">
+        <v>2142</v>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="F11" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_away</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="n">
+        <v>2142</v>
+      </c>
+      <c r="E12" s="2" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="F12" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_away</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="n">
+        <v>2142</v>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>99.20999999999999</v>
+      </c>
+      <c r="F13" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_home</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="n">
+        <v>2143</v>
+      </c>
+      <c r="E14" s="2" t="n">
+        <v>99.26000000000001</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_home</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="n">
+        <v>2143</v>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>99.26000000000001</v>
+      </c>
+      <c r="F15" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_home</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="n">
+        <v>2143</v>
+      </c>
+      <c r="E16" s="2" t="n">
+        <v>99.26000000000001</v>
+      </c>
+      <c r="F16" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>travel_miles_diff</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="n">
+        <v>2154</v>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>99.77</v>
+      </c>
+      <c r="F17" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>altitude_home</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="n">
+        <v>2154</v>
+      </c>
+      <c r="E18" s="2" t="n">
+        <v>99.77</v>
+      </c>
+      <c r="F18" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>elo_diff</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n">
+        <v>2159</v>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F19" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>div_game</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Game-level flag/context</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Game-level</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="n">
+        <v>2159</v>
+      </c>
+      <c r="E20" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F20" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>prime_time</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Game-level flag/context</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Game-level</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="n">
+        <v>2159</v>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F21" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>elo_home</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="n">
+        <v>2159</v>
+      </c>
+      <c r="E22" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F22" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>elo_away</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>2159</v>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F23" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>is_home</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>2159</v>
+      </c>
+      <c r="E24" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="F24" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00808080"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="60" customWidth="1" min="2" max="2"/>
+    <col width="80" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="5" max="5"/>
+    <col width="40" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Plain-English Description</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Definition</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Point-in-time rule</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Missing-value policy</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>altitude_home</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Game-venue elevation in feet</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>altitude_ft of the game stadium</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>venue attribute known before kickoff</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>NaN when the venue is missing from the table</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>committed nfl_stadiums.csv (SRTM/Open-Elevation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>div_game</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Division matchup flag</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>1.0 when home and away share a division else 0.0</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>known before kickoff</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>NaN when the source field is missing</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedule div_game field</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>elo_away</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Away team's pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>team Elo entering kickoff (away side of elo_diff)</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>rating entering kickoff; updated only AFTER a game settles</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>ELO_PRIOR (1500) for a team's first-ever game; never NaN</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedules (all decided REG games, 2018 warmup onward)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>elo_diff</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>elo_home_entering - elo_away_entering; Elo update r += K*(actual - expected), expected = 1/(1+10**((r_opp - r_self)/400)); actual = 1 win / 0 loss / 0.5 tie</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>rating entering kickoff; updated only AFTER a game settles</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>ELO_PRIOR (1500) for a team's first-ever game; never NaN</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedules (all decided REG games, 2018 warmup onward)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>elo_home</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Home team's pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>team Elo entering kickoff (home side of elo_diff)</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>rating entering kickoff; updated only AFTER a game settles</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>ELO_PRIOR (1500) for a team's first-ever game; never NaN</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedules (all decided REG games, 2018 warmup onward)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_away</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Away team's exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>ewm(halflife=2).mean() of the team's net points (for - against) over strictly-prior games</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>per-team ewm over prior games then shift(1)</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>NaN when the team has no prior games</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>decided game scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_diff</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>ewm(halflife=2).mean() of the team's net points (for - against) over strictly-prior games</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>per-team ewm over prior games then shift(1)</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>NaN when the team has no prior games</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>decided game scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_home</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Home team's exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>ewm(halflife=2).mean() of the team's net points (for - against) over strictly-prior games</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>per-team ewm over prior games then shift(1)</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>NaN when the team has no prior games</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>decided game scores</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_away</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Away team's exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>ewm(halflife=2).mean() of the team's game-level yards_gained/n_plays over strictly-prior games</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>per-team ewm over prior games then shift(1)</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>NaN when no prior games or PBP unavailable for a season</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>nflverse play-by-play</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_diff</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>ewm(halflife=2).mean() of the team's game-level yards_gained/n_plays over strictly-prior games</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>per-team ewm over prior games then shift(1)</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>NaN when no prior games or PBP unavailable for a season</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>nflverse play-by-play</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_home</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Home team's exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>ewm(halflife=2).mean() of the team's game-level yards_gained/n_plays over strictly-prior games</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>per-team ewm over prior games then shift(1)</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>NaN when no prior games or PBP unavailable for a season</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>nflverse play-by-play</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>is_dome_home</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Home venue roof is a dome (or closed retractable)</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>1.0 if roof in {dome, closed}; 0.0 if outdoors; NaN unknown</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>venue attribute known before kickoff</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>NaN when roof is unknown/unlisted (e.g. international sites); never fabricated</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedule roof field</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>is_home</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Constant 1.0 anchor for the home-field edge</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>constant 1.0 on every row</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>structural — no data dependency</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>never missing</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>structural constant</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>pace_plays_min_diff</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away trailing plays per minute</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>trailing 4-game mean of n_plays/elapsed_min per game</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>per-team rolling(4).mean().shift(1)</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>NaN when prior games lack clock data</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>nflverse play-by-play clock</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>prime_time</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Evening-kickoff flag</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>1.0 when ET kickoff hour &gt;= 17 else 0.0</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>schedule fact known before kickoff</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>NaN when gametime is missing</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedule gametime (ET)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_away</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Away team's days since its previous game</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>(gameday_t - gameday_{t-1}).days for the away team</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>days since the team's own strictly-prior game</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>NaN for a team's first game of the window; in-model handling</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_diff</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away days since each team's previous game</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>(gameday_t - gameday_{t-1}).days per team</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>days since the team's own strictly-prior game</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>NaN for a team's first game of the window; in-model handling</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_home</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Home team's days since its previous game</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>(gameday_t - gameday_{t-1}).days for the home team</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>days since the team's own strictly-prior game</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>NaN for a team's first game of the window; in-model handling</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>rest_short_diff</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away short-rest flag (rest &lt; 7 days)</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>1.0 when rest_days &lt; 7 else 0.0; home flag minus away flag</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>function of the team's strictly-prior game date</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>NaN when either team has no prior game</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>nflverse schedules</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>travel_miles_diff</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away distance traveled to the venue (miles)</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>haversine(team home stadium, game stadium) home minus away; earth radius 3958.8 mi</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>venue geography, known before kickoff</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>NaN when a stadium is missing from the table; never fabricated</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>committed nfl_stadiums.csv (real coordinates) + nflverse stadium names</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_away</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Away team's trailing win percentage</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>mean(team_win) over the away team's prior 12 games (ties = 0.5)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>per-team rolling(12).mean().shift(1) — current and future games excluded</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>NaN when the team has no prior games; in-model handling</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>decided game outcomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_diff</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away trailing win percentage</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>mean(team_win) over the team's prior 12 games (ties = 0.5)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>per-team rolling(12).mean().shift(1) — current and future games excluded</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>NaN when the team has no prior games; in-model handling</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>decided game outcomes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_home</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Home team's trailing win percentage</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>mean(team_win) over the home team's prior 12 games (ties = 0.5)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>per-team rolling(12).mean().shift(1) — current and future games excluded</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>NaN when the team has no prior games; in-model handling</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>decided game outcomes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="21" customWidth="1" min="1" max="1"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>feature</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>role</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>tested_in_trace</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>elo_diff</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_diff</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_diff</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>is_dome_home</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_diff</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_diff</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>pace_plays_min_diff</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>rest_short_diff</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>div_game</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>travel_miles_diff</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>altitude_home</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>prime_time</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>elo_home</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>elo_away</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_home</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_away</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_home</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_away</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_home</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_away</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_home</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_away</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>is_home</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>production contract</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="b">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -542,6 +2365,2403 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="00808080"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B19"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="90" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>NFL Feature Selection Decision Workbook</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Trace</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>nfl_feature_selection_20260924.json</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Trace schema</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>nfl-rfe-v2</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Run date</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Run mode</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>full_history</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Scoring population (games)</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>2159</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Production width before run</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Candidate pool size</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Full validation pool</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Trials scored</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Committed trials</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Failed trials</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Selected columns (record-only)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>elo_diff, win_pct_diff, rest_days_diff, is_dome_home, ewm_net_pts_diff, ewm_ypp_diff, pace_plays_min_diff, rest_short_diff, div_game, travel_miles_diff, altitude_home, prime_time, elo_home, elo_away, win_pct_home, win_pct_away, ewm_net_pts_home, ewm_net_pts_away, ewm_ypp_home, ewm_ypp_away, rest_days_home, rest_days_away, is_home</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Default governance: this workbook does not change production. Adoption is explicit.</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Commit rule: a trial commits only when its paired log-loss gain clears max(0.0005, 2 x paired SE) with AUC and ECE guardrails.</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Baseline log-loss</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="n">
+        <v>0.6477273264731944</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Best log-loss reached</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>0.6477273264731944</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="002E75B6"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>RFE Run Dashboard</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="n"/>
+      <c r="C1" s="1" t="n"/>
+      <c r="D1" s="1" t="n"/>
+      <c r="E1" s="1" t="n"/>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n"/>
+      <c r="D3" s="2" t="n"/>
+      <c r="E3" s="2" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Trials scored</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C4" s="2" t="n"/>
+      <c r="D4" s="2" t="n"/>
+      <c r="E4" s="2" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C5" s="2" t="n"/>
+      <c r="D5" s="2" t="n"/>
+      <c r="E5" s="2" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Committed removals</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C6" s="2" t="n"/>
+      <c r="D6" s="2" t="n"/>
+      <c r="E6" s="2" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Committed additions</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="2" t="n"/>
+      <c r="D7" s="2" t="n"/>
+      <c r="E7" s="2" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Failed trials (recorded, non-fatal)</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="C8" s="2" t="n"/>
+      <c r="D8" s="2" t="n"/>
+      <c r="E8" s="2" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Features selected (record-only)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="C9" s="2" t="n"/>
+      <c r="D9" s="2" t="n"/>
+      <c r="E9" s="2" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Baseline log-loss</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0.6477273264731944</v>
+      </c>
+      <c r="C10" s="2" t="n"/>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" s="2" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Best log-loss</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>0.6477273264731944</v>
+      </c>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+      <c r="E11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Baseline AUC</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>0.6761755800772</v>
+      </c>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
+      <c r="E12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Best AUC</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>0.6761755800772</v>
+      </c>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
+      <c r="E13" s="2" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Redundant pairs (|r| &gt;= 0.9)</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C14" s="2" t="n"/>
+      <c r="D14" s="2" t="n"/>
+      <c r="E14" s="2" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="n"/>
+      <c r="B15" s="2" t="n"/>
+      <c r="C15" s="2" t="n"/>
+      <c r="D15" s="2" t="n"/>
+      <c r="E15" s="2" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Committed changes this run</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n"/>
+      <c r="C16" s="2" t="n"/>
+      <c r="D16" s="2" t="n"/>
+      <c r="E16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Step</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Log-loss gain</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Committed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00548235"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>In Production</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Plain-English Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>elo_diff</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>full history (iterative)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_diff</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away trailing win percentage</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>12 games</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_diff</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away days since each team's previous game</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>1 games</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>is_dome_home</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Home venue roof is a dome (or closed retractable)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_diff</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_diff</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>pace_plays_min_diff</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away trailing plays per minute</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>4 games</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>rest_short_diff</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away short-rest flag (rest &lt; 7 days)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>1 games</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>div_game</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Game-level flag/context</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Schedule / venue</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Game-level</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Division matchup flag</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>travel_miles_diff</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away distance traveled to the venue (miles)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>altitude_home</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Game-venue elevation in feet</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>prime_time</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Game-level flag/context</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Schedule / venue</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Game-level</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Evening-kickoff flag</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>elo_home</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Home team's pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>full history (iterative)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>elo_away</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Away team's pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>full history (iterative)</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_home</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Home team's trailing win percentage</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>12 games</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_away</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Away team's trailing win percentage</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>12 games</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_home</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Home team's exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_away</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Away team's exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_home</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Home team's exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_away</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Away team's exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_home</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Home team's days since its previous game</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>1 games</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_away</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Away team's days since its previous game</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>1 games</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>is_home</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Constant 1.0 anchor for the home-field edge</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00375623"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>In Production</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Plain-English Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>elo_diff</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>full history (iterative)</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_diff</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away trailing win percentage</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>12 games</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_diff</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away days since each team's previous game</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>1 games</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>is_dome_home</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Home venue roof is a dome (or closed retractable)</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_diff</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_diff</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>pace_plays_min_diff</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away trailing plays per minute</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>4 games</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>rest_short_diff</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away short-rest flag (rest &lt; 7 days)</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>1 games</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>div_game</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Game-level flag/context</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Schedule / venue</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Game-level</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Division matchup flag</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>travel_miles_diff</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Diff</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Team form</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Home − Away (diff)</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Home minus away distance traveled to the venue (miles)</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>altitude_home</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Game-venue elevation in feet</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>prime_time</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Game-level flag/context</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Schedule / venue</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Game-level</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Evening-kickoff flag</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>elo_home</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Home team's pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>full history (iterative)</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>elo_away</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Away team's pre-game Elo rating</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>full history (iterative)</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_home</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Home team's trailing win percentage</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>12 games</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>win_pct_away</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>Away team's trailing win percentage</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>12 games</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_home</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Home team's exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ewm_net_pts_away</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Away team's exponentially-weighted net points per game</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_home</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Home team's exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ewm_ypp_away</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Away team's exponentially-weighted net yards per play</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>decaying (halflife=2 games)</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_home</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Home team's days since its previous game</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>1 games</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>rest_days_away</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Away</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>Away team's days since its previous game</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>1 games</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>is_home</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Raw level (per side)</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>Matchup context</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>Home</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>Constant 1.0 anchor for the home-field edge</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>static pre-game</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="00C55A11"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="80" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="24" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>In Production</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Side</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Plain-English Description</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Window</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Units</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Role in run</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="007030A0"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -1549,9 +5769,10 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="009E5EB5"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
@@ -46867,380 +51088,62 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="002F8F83"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:D2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="21" customWidth="1" min="1" max="1"/>
-    <col width="21" customWidth="1" min="2" max="2"/>
-    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="52" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>feature</t>
+          <t>Feature A</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>role</t>
+          <t>Feature B</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>tested_in_trace</t>
+          <t>Pearson r</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>elo_diff</t>
+          <t>rest_days_home</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C2" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>win_pct_diff</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>rest_days_diff</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>is_dome_home</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C5" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>ewm_net_pts_diff</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C6" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>ewm_ypp_diff</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>pace_plays_min_diff</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C8" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>rest_short_diff</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C9" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>div_game</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="inlineStr">
-        <is>
-          <t>travel_miles_diff</t>
-        </is>
-      </c>
-      <c r="B11" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C11" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>altitude_home</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>prime_time</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>elo_home</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>elo_away</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>win_pct_home</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>win_pct_away</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>ewm_net_pts_home</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>ewm_net_pts_away</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>ewm_ypp_home</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>ewm_ypp_away</t>
-        </is>
-      </c>
-      <c r="B21" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C21" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="2" t="inlineStr">
-        <is>
-          <t>rest_days_home</t>
-        </is>
-      </c>
-      <c r="B22" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C22" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
           <t>rest_days_away</t>
         </is>
       </c>
-      <c r="B23" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>is_home</t>
-        </is>
-      </c>
-      <c r="B24" s="2" t="inlineStr">
-        <is>
-          <t>production contract</t>
-        </is>
-      </c>
-      <c r="C24" s="2" t="b">
-        <v>1</v>
+      <c r="C2" s="2" t="n">
+        <v>0.9991</v>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>near-duplicate signal — consider one representative</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>